<commit_message>
WS2812B led alternate added
</commit_message>
<xml_diff>
--- a/Design Files/Catan_Board/Secondary_PCB/BOM/JLCPCB BOM.xlsx
+++ b/Design Files/Catan_Board/Secondary_PCB/BOM/JLCPCB BOM.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\jakekrum-catanboard\Design Files\Catan_Board\Secondary_PCB\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Faizan\GitHub\jakekrum-catanboard\Design Files\Catan_Board\Secondary_PCB\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D35037B-8698-4C79-9BA1-FDC40B33C225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Comment</t>
   </si>
@@ -60,13 +61,16 @@
     <t>C160316</t>
   </si>
   <si>
-    <t>C114586</t>
+    <t>WS2812B-B/T</t>
+  </si>
+  <si>
+    <t>C2761795</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -504,18 +508,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -529,7 +533,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -543,7 +547,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
@@ -557,7 +561,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -565,10 +569,10 @@
         <v>7</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>